<commit_message>
Remove answer-control language and refresh Windows evidence
</commit_message>
<xml_diff>
--- a/artifacts/任务规格转化.xlsx
+++ b/artifacts/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="Raf4587ced6854f5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R7b4aa2c5842d457d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -466,7 +466,7 @@
         <x:v>发布路径关系</x:v>
       </x:c>
       <x:c r="B14" s="21" t="str">
-        <x:v>tenant_release_matrix.csv按tenant_id与flag_key唯一定位配置，config_path从reference.zip根目录书写，摘要中的config_files与矩阵集合一致</x:v>
+        <x:v>tenant_release_matrix.csv按tenant_id与flag_key唯一定位配置，config_path以output/configs为前缀并指向正式交付目录中的实际文件，摘要中的config_files与矩阵集合一致</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="56" customHeight="1">
@@ -474,7 +474,7 @@
         <x:v>失败收口</x:v>
       </x:c>
       <x:c r="B15" s="21" t="str">
-        <x:v>patch_queue.jsonl无法完整解析或候选源码非零退出时不发布本轮reports和configs；输入文件保持只读</x:v>
+        <x:v>patch_queue.jsonl无法完整解析或发布编排源码非零退出时不发布本轮reports和configs；输入文件保持只读</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="54" customHeight="1">

</xml_diff>